<commit_message>
Fix battery MLF gaps: include BIDIRECTIONAL dispatch type in DUDETAILSUMMARY filter
AEMO migrated batteries from separate GENERATOR G-suffix DUIDs (e.g. HPRG1, VBBG1)
to single BIDIRECTIONAL registration DUIDs (e.g. HPR1, VBB1) during 2024. The
existing filter (DISPATCHTYPE == 'GENERATOR') silently excluded all post-migration
battery records, causing:
  - Data ending at FY24-25 for batteries that transitioned
  - FY25-26 gaps across the board for batteries
  - Stub rows covering 69 DUIDs (now only 9 genuinely new assets)

Fix: include BIDIRECTIONAL in the dispatch type filter.

Result: FY-level extraction yields 727 DUIDs with history (was 667); stub rows
drop from 69 → 9 (only genuinely new/pre-operational assets remain as stubs).
</commit_message>
<xml_diff>
--- a/outputs/QLD_mlf.xlsx
+++ b/outputs/QLD_mlf.xlsx
@@ -1024,12 +1024,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>KSP1</t>
+          <t>HUGSF1</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Kidston Solar Project Phase One</t>
+          <t>Hughenden Solar Farm</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1038,12 +1038,12 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>50</v>
+        <v>20.97</v>
       </c>
       <c r="E10" s="4" t="inlineStr"/>
       <c r="F10" s="4" t="inlineStr"/>
       <c r="G10" s="4" t="n">
-        <v>1.0149</v>
+        <v>1.0115</v>
       </c>
       <c r="H10" s="4" t="n">
         <v>0.8842</v>
@@ -1140,12 +1140,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>HUGSF1</t>
+          <t>KSP1</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Hughenden Solar Farm</t>
+          <t>Kidston Solar Project Phase One</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1154,12 +1154,12 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>20.97</v>
+        <v>50</v>
       </c>
       <c r="E12" s="4" t="inlineStr"/>
       <c r="F12" s="4" t="inlineStr"/>
       <c r="G12" s="4" t="n">
-        <v>1.0115</v>
+        <v>1.0149</v>
       </c>
       <c r="H12" s="4" t="n">
         <v>0.8842</v>
@@ -1354,12 +1354,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>LRSF1</t>
+          <t>CLERMSF1</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Longreach Solar Farm</t>
+          <t>Clermont Solar Farm</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1368,15 +1368,13 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>17</v>
+        <v>92.5</v>
       </c>
       <c r="E16" s="4" t="inlineStr"/>
       <c r="F16" s="4" t="inlineStr"/>
-      <c r="G16" s="4" t="n">
-        <v>0.9689</v>
-      </c>
+      <c r="G16" s="4" t="inlineStr"/>
       <c r="H16" s="4" t="n">
-        <v>0.8934</v>
+        <v>0.8862</v>
       </c>
       <c r="I16" s="4" t="n">
         <v>0.8735000000000001</v>
@@ -1472,12 +1470,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>CLERMSF1</t>
+          <t>LRSF1</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Clermont Solar Farm</t>
+          <t>Longreach Solar Farm</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1486,13 +1484,15 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>92.5</v>
+        <v>17</v>
       </c>
       <c r="E18" s="4" t="inlineStr"/>
       <c r="F18" s="4" t="inlineStr"/>
-      <c r="G18" s="4" t="inlineStr"/>
+      <c r="G18" s="4" t="n">
+        <v>0.9689</v>
+      </c>
       <c r="H18" s="4" t="n">
-        <v>0.8862</v>
+        <v>0.8934</v>
       </c>
       <c r="I18" s="4" t="n">
         <v>0.8735000000000001</v>
@@ -1737,13 +1737,21 @@
       <c r="K23" s="4" t="inlineStr"/>
       <c r="L23" s="4" t="inlineStr"/>
       <c r="M23" s="4" t="inlineStr"/>
-      <c r="N23" s="4" t="inlineStr"/>
-      <c r="O23" s="4" t="inlineStr"/>
+      <c r="N23" s="4" t="n">
+        <v>0.9528</v>
+      </c>
+      <c r="O23" s="4" t="n">
+        <v>0.9358</v>
+      </c>
       <c r="P23" s="4" t="n">
         <v>0.9008</v>
       </c>
-      <c r="Q23" s="4" t="inlineStr"/>
-      <c r="R23" s="5" t="inlineStr"/>
+      <c r="Q23" s="4" t="n">
+        <v>-0.035</v>
+      </c>
+      <c r="R23" s="5" t="n">
+        <v>-3.74</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2058,12 +2066,12 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>OAKY2</t>
+          <t>OAKYCREK</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Oaky Creek 2</t>
+          <t>Oaky Creek Power Station</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -2072,7 +2080,7 @@
         </is>
       </c>
       <c r="D29" s="3" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E29" s="4" t="n">
         <v>1.0373</v>
@@ -2120,12 +2128,12 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>OAKYCREK</t>
+          <t>OAKY2</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Oaky Creek Power Station</t>
+          <t>Oaky Creek 2</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -2134,7 +2142,7 @@
         </is>
       </c>
       <c r="D30" s="3" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="E30" s="4" t="n">
         <v>1.0373</v>
@@ -2182,7 +2190,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>CALL_A_4</t>
+          <t>CALLNL4</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -2190,11 +2198,7 @@
           <t>Callide Power Station</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>Fossil</t>
-        </is>
-      </c>
+      <c r="C31" s="2" t="inlineStr"/>
       <c r="D31" s="3" t="n">
         <v>30</v>
       </c>
@@ -2232,7 +2236,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>CALLNL4</t>
+          <t>CALL_A_4</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -2240,7 +2244,11 @@
           <t>Callide Power Station</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr"/>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Fossil</t>
+        </is>
+      </c>
       <c r="D32" s="3" t="n">
         <v>30</v>
       </c>
@@ -2278,7 +2286,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>STAN-3</t>
+          <t>STAN-1</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -2402,7 +2410,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>STAN-1</t>
+          <t>STAN-3</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -2774,7 +2782,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>BRDDSF01</t>
+          <t>BRDDBES1</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -2784,11 +2792,11 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Solar</t>
+          <t>Battery</t>
         </is>
       </c>
       <c r="D41" s="3" t="n">
-        <v>368</v>
+        <v>240</v>
       </c>
       <c r="E41" s="4" t="inlineStr"/>
       <c r="F41" s="4" t="inlineStr"/>
@@ -2816,7 +2824,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>BRDDBES1</t>
+          <t>BRDDSF01</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -2826,11 +2834,11 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Battery</t>
+          <t>Solar</t>
         </is>
       </c>
       <c r="D42" s="3" t="n">
-        <v>240</v>
+        <v>368</v>
       </c>
       <c r="E42" s="4" t="inlineStr"/>
       <c r="F42" s="4" t="inlineStr"/>
@@ -2842,12 +2850,18 @@
       <c r="L42" s="4" t="inlineStr"/>
       <c r="M42" s="4" t="inlineStr"/>
       <c r="N42" s="4" t="inlineStr"/>
-      <c r="O42" s="4" t="inlineStr"/>
+      <c r="O42" s="4" t="n">
+        <v>0.929</v>
+      </c>
       <c r="P42" s="4" t="n">
         <v>0.9247</v>
       </c>
-      <c r="Q42" s="4" t="inlineStr"/>
-      <c r="R42" s="5" t="inlineStr"/>
+      <c r="Q42" s="4" t="n">
+        <v>-0.0043</v>
+      </c>
+      <c r="R42" s="5" t="n">
+        <v>-0.46</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3100,7 +3114,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>GSTONE6</t>
+          <t>GSTONE5</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -3162,7 +3176,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>GSTONE5</t>
+          <t>GSTONE6</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -3812,12 +3826,12 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>SRSF1</t>
+          <t>CHILDSF1</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Susan River Solar Farm</t>
+          <t>Childers Solar Farm</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -3826,7 +3840,7 @@
         </is>
       </c>
       <c r="D60" s="3" t="n">
-        <v>85.26000000000001</v>
+        <v>64.38</v>
       </c>
       <c r="E60" s="4" t="inlineStr"/>
       <c r="F60" s="4" t="inlineStr"/>
@@ -3868,12 +3882,12 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>CHILDSF1</t>
+          <t>SRSF1</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Childers Solar Farm</t>
+          <t>Susan River Solar Farm</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -3882,7 +3896,7 @@
         </is>
       </c>
       <c r="D61" s="3" t="n">
-        <v>64.38</v>
+        <v>85.26000000000001</v>
       </c>
       <c r="E61" s="4" t="inlineStr"/>
       <c r="F61" s="4" t="inlineStr"/>
@@ -3986,7 +4000,7 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>MSTUART3</t>
+          <t>MSTUART2</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -4000,7 +4014,7 @@
         </is>
       </c>
       <c r="D63" s="3" t="n">
-        <v>131</v>
+        <v>144</v>
       </c>
       <c r="E63" s="4" t="n">
         <v>1.0156</v>
@@ -4048,7 +4062,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>MSTUART2</t>
+          <t>MSTUART3</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -4062,7 +4076,7 @@
         </is>
       </c>
       <c r="D64" s="3" t="n">
-        <v>144</v>
+        <v>131</v>
       </c>
       <c r="E64" s="4" t="n">
         <v>1.0156</v>
@@ -4394,7 +4408,7 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>KAREEYA4</t>
+          <t>KAREEYA2</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -4456,7 +4470,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>KAREEYA1</t>
+          <t>KAREEYA5</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -4470,7 +4484,7 @@
         </is>
       </c>
       <c r="D72" s="3" t="n">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="E72" s="4" t="n">
         <v>1.069</v>
@@ -4518,7 +4532,7 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>KAREEYA2</t>
+          <t>KAREEYA4</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -4642,7 +4656,7 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>KAREEYA5</t>
+          <t>KAREEYA1</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -4656,7 +4670,7 @@
         </is>
       </c>
       <c r="D75" s="3" t="n">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="E75" s="4" t="n">
         <v>1.069</v>
@@ -4990,12 +5004,12 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>BRAEMAR6</t>
+          <t>BRAEMAR2</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>Braemar 2 Power Station</t>
+          <t>Braemar Power Station</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
@@ -5004,7 +5018,7 @@
         </is>
       </c>
       <c r="D81" s="3" t="n">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="E81" s="4" t="n">
         <v>0.9567</v>
@@ -5114,12 +5128,12 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>BRAEMAR1</t>
+          <t>BRAEMAR7</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>Braemar Power Station</t>
+          <t>Braemar 2 Power Station</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
@@ -5128,7 +5142,7 @@
         </is>
       </c>
       <c r="D83" s="3" t="n">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="E83" s="4" t="n">
         <v>0.9567</v>
@@ -5176,12 +5190,12 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>BRAEMAR2</t>
+          <t>BRAEMAR6</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>Braemar Power Station</t>
+          <t>Braemar 2 Power Station</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
@@ -5190,7 +5204,7 @@
         </is>
       </c>
       <c r="D84" s="3" t="n">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="E84" s="4" t="n">
         <v>0.9567</v>
@@ -5238,12 +5252,12 @@
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>BRAEMAR7</t>
+          <t>BRAEMAR1</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>Braemar 2 Power Station</t>
+          <t>Braemar Power Station</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
@@ -5252,7 +5266,7 @@
         </is>
       </c>
       <c r="D85" s="3" t="n">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="E85" s="4" t="n">
         <v>0.9567</v>
@@ -5530,7 +5544,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>TARONG#4</t>
+          <t>TARONG#3</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -5592,7 +5606,7 @@
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>TARONG#3</t>
+          <t>TARONG#4</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
@@ -5977,13 +5991,21 @@
       <c r="K97" s="4" t="inlineStr"/>
       <c r="L97" s="4" t="inlineStr"/>
       <c r="M97" s="4" t="inlineStr"/>
-      <c r="N97" s="4" t="inlineStr"/>
-      <c r="O97" s="4" t="inlineStr"/>
+      <c r="N97" s="4" t="n">
+        <v>0.9837</v>
+      </c>
+      <c r="O97" s="4" t="n">
+        <v>0.9836</v>
+      </c>
       <c r="P97" s="4" t="n">
         <v>0.9772999999999999</v>
       </c>
-      <c r="Q97" s="4" t="inlineStr"/>
-      <c r="R97" s="5" t="inlineStr"/>
+      <c r="Q97" s="4" t="n">
+        <v>-0.0063</v>
+      </c>
+      <c r="R97" s="5" t="n">
+        <v>-0.64</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -6050,7 +6072,7 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>ROMA_7</t>
+          <t>ROMA_8</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
@@ -6112,7 +6134,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>ROMA_8</t>
+          <t>ROMA_7</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -6199,13 +6221,21 @@
       <c r="K101" s="4" t="inlineStr"/>
       <c r="L101" s="4" t="inlineStr"/>
       <c r="M101" s="4" t="inlineStr"/>
-      <c r="N101" s="4" t="inlineStr"/>
-      <c r="O101" s="4" t="inlineStr"/>
+      <c r="N101" s="4" t="n">
+        <v>0.9698</v>
+      </c>
+      <c r="O101" s="4" t="n">
+        <v>0.9851</v>
+      </c>
       <c r="P101" s="4" t="n">
         <v>0.9778</v>
       </c>
-      <c r="Q101" s="4" t="inlineStr"/>
-      <c r="R101" s="5" t="inlineStr"/>
+      <c r="Q101" s="4" t="n">
+        <v>-0.0073</v>
+      </c>
+      <c r="R101" s="5" t="n">
+        <v>-0.74</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -6235,13 +6265,21 @@
       <c r="K102" s="4" t="inlineStr"/>
       <c r="L102" s="4" t="inlineStr"/>
       <c r="M102" s="4" t="inlineStr"/>
-      <c r="N102" s="4" t="inlineStr"/>
-      <c r="O102" s="4" t="inlineStr"/>
+      <c r="N102" s="4" t="n">
+        <v>0.9761</v>
+      </c>
+      <c r="O102" s="4" t="n">
+        <v>0.9875</v>
+      </c>
       <c r="P102" s="4" t="n">
         <v>0.9787</v>
       </c>
-      <c r="Q102" s="4" t="inlineStr"/>
-      <c r="R102" s="5" t="inlineStr"/>
+      <c r="Q102" s="4" t="n">
+        <v>-0.008800000000000001</v>
+      </c>
+      <c r="R102" s="5" t="n">
+        <v>-0.89</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -6642,12 +6680,12 @@
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>WDBESS1</t>
+          <t>WDBESS2</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>Western Downs Battery Energy Storage System</t>
+          <t>Western Downs Battery Energy Storage System (BESS)</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
@@ -6656,7 +6694,7 @@
         </is>
       </c>
       <c r="D110" s="3" t="n">
-        <v>272.48</v>
+        <v>269.8</v>
       </c>
       <c r="E110" s="4" t="inlineStr"/>
       <c r="F110" s="4" t="inlineStr"/>
@@ -6668,22 +6706,28 @@
       <c r="L110" s="4" t="inlineStr"/>
       <c r="M110" s="4" t="inlineStr"/>
       <c r="N110" s="4" t="inlineStr"/>
-      <c r="O110" s="4" t="inlineStr"/>
+      <c r="O110" s="4" t="n">
+        <v>0.9899</v>
+      </c>
       <c r="P110" s="4" t="n">
         <v>0.9801</v>
       </c>
-      <c r="Q110" s="4" t="inlineStr"/>
-      <c r="R110" s="5" t="inlineStr"/>
+      <c r="Q110" s="4" t="n">
+        <v>-0.0098</v>
+      </c>
+      <c r="R110" s="5" t="n">
+        <v>-0.99</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>WDBESS2</t>
+          <t>WDBESS1</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>Western Downs Battery Energy Storage System (BESS)</t>
+          <t>Western Downs Battery Energy Storage System</t>
         </is>
       </c>
       <c r="C111" s="2" t="inlineStr">
@@ -6692,7 +6736,7 @@
         </is>
       </c>
       <c r="D111" s="3" t="n">
-        <v>269.8</v>
+        <v>272.48</v>
       </c>
       <c r="E111" s="4" t="inlineStr"/>
       <c r="F111" s="4" t="inlineStr"/>
@@ -6703,13 +6747,21 @@
       <c r="K111" s="4" t="inlineStr"/>
       <c r="L111" s="4" t="inlineStr"/>
       <c r="M111" s="4" t="inlineStr"/>
-      <c r="N111" s="4" t="inlineStr"/>
-      <c r="O111" s="4" t="inlineStr"/>
+      <c r="N111" s="4" t="n">
+        <v>0.9762</v>
+      </c>
+      <c r="O111" s="4" t="n">
+        <v>0.9891</v>
+      </c>
       <c r="P111" s="4" t="n">
         <v>0.9801</v>
       </c>
-      <c r="Q111" s="4" t="inlineStr"/>
-      <c r="R111" s="5" t="inlineStr"/>
+      <c r="Q111" s="4" t="n">
+        <v>-0.008999999999999999</v>
+      </c>
+      <c r="R111" s="5" t="n">
+        <v>-0.91</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -7152,60 +7204,66 @@
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>DULAWF1</t>
+          <t>MARYRSF1</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>Dulacca Wind Farm</t>
+          <t>Maryrorough Solar Farm</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>Wind</t>
+          <t>Solar</t>
         </is>
       </c>
       <c r="D120" s="3" t="n">
-        <v>180</v>
+        <v>33</v>
       </c>
       <c r="E120" s="4" t="inlineStr"/>
       <c r="F120" s="4" t="inlineStr"/>
       <c r="G120" s="4" t="inlineStr"/>
       <c r="H120" s="4" t="inlineStr"/>
-      <c r="I120" s="4" t="inlineStr"/>
-      <c r="J120" s="4" t="inlineStr"/>
-      <c r="K120" s="4" t="inlineStr"/>
+      <c r="I120" s="4" t="n">
+        <v>0.9872</v>
+      </c>
+      <c r="J120" s="4" t="n">
+        <v>0.9851</v>
+      </c>
+      <c r="K120" s="4" t="n">
+        <v>0.9789</v>
+      </c>
       <c r="L120" s="4" t="n">
-        <v>0.9540999999999999</v>
+        <v>0.9861</v>
       </c>
       <c r="M120" s="4" t="n">
-        <v>0.9776</v>
+        <v>0.9913999999999999</v>
       </c>
       <c r="N120" s="4" t="n">
-        <v>0.977</v>
+        <v>0.9847</v>
       </c>
       <c r="O120" s="4" t="n">
-        <v>0.9853</v>
+        <v>0.9888</v>
       </c>
       <c r="P120" s="4" t="n">
         <v>0.987</v>
       </c>
       <c r="Q120" s="4" t="n">
-        <v>0.0017</v>
+        <v>-0.0018</v>
       </c>
       <c r="R120" s="5" t="n">
-        <v>0.17</v>
+        <v>-0.18</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>MARYRSF1</t>
+          <t>WARWSF1</t>
         </is>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>Maryrorough Solar Farm</t>
+          <t xml:space="preserve">Warwick Solar Farm 1 </t>
         </is>
       </c>
       <c r="C121" s="2" t="inlineStr">
@@ -7214,15 +7272,13 @@
         </is>
       </c>
       <c r="D121" s="3" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="E121" s="4" t="inlineStr"/>
       <c r="F121" s="4" t="inlineStr"/>
       <c r="G121" s="4" t="inlineStr"/>
       <c r="H121" s="4" t="inlineStr"/>
-      <c r="I121" s="4" t="n">
-        <v>0.9872</v>
-      </c>
+      <c r="I121" s="4" t="inlineStr"/>
       <c r="J121" s="4" t="n">
         <v>0.9851</v>
       </c>
@@ -7254,53 +7310,49 @@
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>WARWSF1</t>
+          <t>DULAWF1</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Warwick Solar Farm 1 </t>
+          <t>Dulacca Wind Farm</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>Solar</t>
+          <t>Wind</t>
         </is>
       </c>
       <c r="D122" s="3" t="n">
-        <v>39</v>
+        <v>180</v>
       </c>
       <c r="E122" s="4" t="inlineStr"/>
       <c r="F122" s="4" t="inlineStr"/>
       <c r="G122" s="4" t="inlineStr"/>
       <c r="H122" s="4" t="inlineStr"/>
       <c r="I122" s="4" t="inlineStr"/>
-      <c r="J122" s="4" t="n">
-        <v>0.9851</v>
-      </c>
-      <c r="K122" s="4" t="n">
-        <v>0.9789</v>
-      </c>
+      <c r="J122" s="4" t="inlineStr"/>
+      <c r="K122" s="4" t="inlineStr"/>
       <c r="L122" s="4" t="n">
-        <v>0.9861</v>
+        <v>0.9540999999999999</v>
       </c>
       <c r="M122" s="4" t="n">
-        <v>0.9913999999999999</v>
+        <v>0.9776</v>
       </c>
       <c r="N122" s="4" t="n">
-        <v>0.9847</v>
+        <v>0.977</v>
       </c>
       <c r="O122" s="4" t="n">
-        <v>0.9888</v>
+        <v>0.9853</v>
       </c>
       <c r="P122" s="4" t="n">
         <v>0.987</v>
       </c>
       <c r="Q122" s="4" t="n">
-        <v>-0.0018</v>
+        <v>0.0017</v>
       </c>
       <c r="R122" s="5" t="n">
-        <v>-0.18</v>
+        <v>0.17</v>
       </c>
     </row>
     <row r="123">
@@ -7644,38 +7696,60 @@
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>SNB02</t>
+          <t>DG_QLD1</t>
         </is>
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t>Supernode BESS</t>
-        </is>
-      </c>
-      <c r="C129" s="2" t="inlineStr">
-        <is>
-          <t>Battery</t>
-        </is>
-      </c>
+          <t>QLD1 Dummy Generator</t>
+        </is>
+      </c>
+      <c r="C129" s="2" t="inlineStr"/>
       <c r="D129" s="3" t="n">
-        <v>337.4</v>
-      </c>
-      <c r="E129" s="4" t="inlineStr"/>
-      <c r="F129" s="4" t="inlineStr"/>
-      <c r="G129" s="4" t="inlineStr"/>
-      <c r="H129" s="4" t="inlineStr"/>
-      <c r="I129" s="4" t="inlineStr"/>
-      <c r="J129" s="4" t="inlineStr"/>
-      <c r="K129" s="4" t="inlineStr"/>
-      <c r="L129" s="4" t="inlineStr"/>
-      <c r="M129" s="4" t="inlineStr"/>
-      <c r="N129" s="4" t="inlineStr"/>
-      <c r="O129" s="4" t="inlineStr"/>
+        <v>3000</v>
+      </c>
+      <c r="E129" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F129" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G129" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H129" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I129" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J129" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K129" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L129" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M129" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N129" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O129" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="P129" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="Q129" s="4" t="inlineStr"/>
-      <c r="R129" s="5" t="inlineStr"/>
+      <c r="Q129" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R129" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -7705,59 +7779,51 @@
       <c r="K130" s="4" t="inlineStr"/>
       <c r="L130" s="4" t="inlineStr"/>
       <c r="M130" s="4" t="inlineStr"/>
-      <c r="N130" s="4" t="inlineStr"/>
-      <c r="O130" s="4" t="inlineStr"/>
+      <c r="N130" s="4" t="n">
+        <v>0.9877</v>
+      </c>
+      <c r="O130" s="4" t="n">
+        <v>1.0066</v>
+      </c>
       <c r="P130" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="Q130" s="4" t="inlineStr"/>
-      <c r="R130" s="5" t="inlineStr"/>
+      <c r="Q130" s="4" t="n">
+        <v>-0.0066</v>
+      </c>
+      <c r="R130" s="5" t="n">
+        <v>-0.66</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>DG_QLD1</t>
+          <t>SNB02</t>
         </is>
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>QLD1 Dummy Generator</t>
-        </is>
-      </c>
-      <c r="C131" s="2" t="inlineStr"/>
+          <t>Supernode BESS</t>
+        </is>
+      </c>
+      <c r="C131" s="2" t="inlineStr">
+        <is>
+          <t>Battery</t>
+        </is>
+      </c>
       <c r="D131" s="3" t="n">
-        <v>3000</v>
-      </c>
-      <c r="E131" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F131" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G131" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H131" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I131" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J131" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K131" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L131" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="M131" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="N131" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>337.4</v>
+      </c>
+      <c r="E131" s="4" t="inlineStr"/>
+      <c r="F131" s="4" t="inlineStr"/>
+      <c r="G131" s="4" t="inlineStr"/>
+      <c r="H131" s="4" t="inlineStr"/>
+      <c r="I131" s="4" t="inlineStr"/>
+      <c r="J131" s="4" t="inlineStr"/>
+      <c r="K131" s="4" t="inlineStr"/>
+      <c r="L131" s="4" t="inlineStr"/>
+      <c r="M131" s="4" t="inlineStr"/>
+      <c r="N131" s="4" t="inlineStr"/>
       <c r="O131" s="4" t="n">
         <v>1</v>
       </c>
@@ -7800,12 +7866,18 @@
       <c r="L132" s="4" t="inlineStr"/>
       <c r="M132" s="4" t="inlineStr"/>
       <c r="N132" s="4" t="inlineStr"/>
-      <c r="O132" s="4" t="inlineStr"/>
+      <c r="O132" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="P132" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="Q132" s="4" t="inlineStr"/>
-      <c r="R132" s="5" t="inlineStr"/>
+      <c r="Q132" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R132" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -7970,12 +8042,18 @@
       <c r="L136" s="4" t="inlineStr"/>
       <c r="M136" s="4" t="inlineStr"/>
       <c r="N136" s="4" t="inlineStr"/>
-      <c r="O136" s="4" t="inlineStr"/>
+      <c r="O136" s="4" t="n">
+        <v>1.0036</v>
+      </c>
       <c r="P136" s="4" t="n">
         <v>1.0015</v>
       </c>
-      <c r="Q136" s="4" t="inlineStr"/>
-      <c r="R136" s="5" t="inlineStr"/>
+      <c r="Q136" s="4" t="n">
+        <v>-0.0021</v>
+      </c>
+      <c r="R136" s="5" t="n">
+        <v>-0.21</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -8130,12 +8208,18 @@
       <c r="L139" s="4" t="inlineStr"/>
       <c r="M139" s="4" t="inlineStr"/>
       <c r="N139" s="4" t="inlineStr"/>
-      <c r="O139" s="4" t="inlineStr"/>
+      <c r="O139" s="4" t="n">
+        <v>1.0014</v>
+      </c>
       <c r="P139" s="4" t="n">
         <v>1.0027</v>
       </c>
-      <c r="Q139" s="4" t="inlineStr"/>
-      <c r="R139" s="5" t="inlineStr"/>
+      <c r="Q139" s="4" t="n">
+        <v>0.0013</v>
+      </c>
+      <c r="R139" s="5" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -8223,13 +8307,21 @@
       <c r="K141" s="4" t="inlineStr"/>
       <c r="L141" s="4" t="inlineStr"/>
       <c r="M141" s="4" t="inlineStr"/>
-      <c r="N141" s="4" t="inlineStr"/>
-      <c r="O141" s="4" t="inlineStr"/>
+      <c r="N141" s="4" t="n">
+        <v>1.0033</v>
+      </c>
+      <c r="O141" s="4" t="n">
+        <v>1.0045</v>
+      </c>
       <c r="P141" s="4" t="n">
         <v>1.0035</v>
       </c>
-      <c r="Q141" s="4" t="inlineStr"/>
-      <c r="R141" s="5" t="inlineStr"/>
+      <c r="Q141" s="4" t="n">
+        <v>-0.001</v>
+      </c>
+      <c r="R141" s="5" t="n">
+        <v>-0.1</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -8296,12 +8388,12 @@
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>RPCG</t>
+          <t>STAPYLTON1</t>
         </is>
       </c>
       <c r="B143" s="2" t="inlineStr">
         <is>
-          <t>Rocky Point Cogeneration Plant</t>
+          <t>Stapylton Renewable Energy Facility</t>
         </is>
       </c>
       <c r="C143" s="2" t="inlineStr">
@@ -8310,14 +8402,10 @@
         </is>
       </c>
       <c r="D143" s="3" t="n">
-        <v>30</v>
-      </c>
-      <c r="E143" s="4" t="n">
-        <v>1.0078</v>
-      </c>
-      <c r="F143" s="4" t="n">
-        <v>1.008</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="E143" s="4" t="inlineStr"/>
+      <c r="F143" s="4" t="inlineStr"/>
       <c r="G143" s="4" t="n">
         <v>1.0112</v>
       </c>
@@ -8358,12 +8446,12 @@
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>STAPYLTON1</t>
+          <t>RPCG</t>
         </is>
       </c>
       <c r="B144" s="2" t="inlineStr">
         <is>
-          <t>Stapylton Renewable Energy Facility</t>
+          <t>Rocky Point Cogeneration Plant</t>
         </is>
       </c>
       <c r="C144" s="2" t="inlineStr">
@@ -8372,10 +8460,14 @@
         </is>
       </c>
       <c r="D144" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E144" s="4" t="inlineStr"/>
-      <c r="F144" s="4" t="inlineStr"/>
+        <v>30</v>
+      </c>
+      <c r="E144" s="4" t="n">
+        <v>1.0078</v>
+      </c>
+      <c r="F144" s="4" t="n">
+        <v>1.008</v>
+      </c>
       <c r="G144" s="4" t="n">
         <v>1.0112</v>
       </c>
@@ -8830,12 +8922,12 @@
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>EDLRGNRD</t>
+          <t>ROCHEDAL</t>
         </is>
       </c>
       <c r="B153" s="2" t="inlineStr">
         <is>
-          <t>Roghan Road LFG Power Plant</t>
+          <t>Rochedale Renewable Energy Facility</t>
         </is>
       </c>
       <c r="C153" s="2" t="inlineStr">
@@ -8844,22 +8936,22 @@
         </is>
       </c>
       <c r="D153" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E153" s="4" t="n">
-        <v>1.0057</v>
+        <v>1.0067</v>
       </c>
       <c r="F153" s="4" t="n">
-        <v>1.0049</v>
+        <v>1.0091</v>
       </c>
       <c r="G153" s="4" t="n">
-        <v>1.0044</v>
+        <v>1.0114</v>
       </c>
       <c r="H153" s="4" t="n">
-        <v>1.0042</v>
+        <v>1.0123</v>
       </c>
       <c r="I153" s="4" t="n">
-        <v>1.0042</v>
+        <v>1.0121</v>
       </c>
       <c r="J153" s="4" t="inlineStr"/>
       <c r="K153" s="4" t="inlineStr"/>
@@ -8874,12 +8966,12 @@
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>ROCHEDAL</t>
+          <t>WHIT1</t>
         </is>
       </c>
       <c r="B154" s="2" t="inlineStr">
         <is>
-          <t>Rochedale Renewable Energy Facility</t>
+          <t>Whitwood Road Renewable Energy Facility</t>
         </is>
       </c>
       <c r="C154" s="2" t="inlineStr">
@@ -8888,22 +8980,22 @@
         </is>
       </c>
       <c r="D154" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E154" s="4" t="n">
-        <v>1.0067</v>
+        <v>0.9953</v>
       </c>
       <c r="F154" s="4" t="n">
-        <v>1.0091</v>
+        <v>0.9968</v>
       </c>
       <c r="G154" s="4" t="n">
-        <v>1.0114</v>
+        <v>0.9999</v>
       </c>
       <c r="H154" s="4" t="n">
-        <v>1.0123</v>
+        <v>1.0001</v>
       </c>
       <c r="I154" s="4" t="n">
-        <v>1.0121</v>
+        <v>1.0006</v>
       </c>
       <c r="J154" s="4" t="inlineStr"/>
       <c r="K154" s="4" t="inlineStr"/>
@@ -8918,12 +9010,12 @@
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>WHIT1</t>
+          <t>EDLRGNRD</t>
         </is>
       </c>
       <c r="B155" s="2" t="inlineStr">
         <is>
-          <t>Whitwood Road Renewable Energy Facility</t>
+          <t>Roghan Road LFG Power Plant</t>
         </is>
       </c>
       <c r="C155" s="2" t="inlineStr">
@@ -8932,22 +9024,22 @@
         </is>
       </c>
       <c r="D155" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E155" s="4" t="n">
-        <v>0.9953</v>
+        <v>1.0057</v>
       </c>
       <c r="F155" s="4" t="n">
-        <v>0.9968</v>
+        <v>1.0049</v>
       </c>
       <c r="G155" s="4" t="n">
-        <v>0.9999</v>
+        <v>1.0044</v>
       </c>
       <c r="H155" s="4" t="n">
-        <v>1.0001</v>
+        <v>1.0042</v>
       </c>
       <c r="I155" s="4" t="n">
-        <v>1.0006</v>
+        <v>1.0042</v>
       </c>
       <c r="J155" s="4" t="inlineStr"/>
       <c r="K155" s="4" t="inlineStr"/>
@@ -9102,12 +9194,12 @@
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>WDBESSG1</t>
+          <t>WANDBG1</t>
         </is>
       </c>
       <c r="B159" s="2" t="inlineStr">
         <is>
-          <t>Western Downs Battery Energy Storage System (BESS)</t>
+          <t>Wandoan BESS</t>
         </is>
       </c>
       <c r="C159" s="2" t="inlineStr">
@@ -9116,7 +9208,7 @@
         </is>
       </c>
       <c r="D159" s="3" t="n">
-        <v>272</v>
+        <v>123</v>
       </c>
       <c r="E159" s="4" t="inlineStr"/>
       <c r="F159" s="4" t="inlineStr"/>
@@ -9124,13 +9216,17 @@
       <c r="H159" s="4" t="inlineStr"/>
       <c r="I159" s="4" t="inlineStr"/>
       <c r="J159" s="4" t="inlineStr"/>
-      <c r="K159" s="4" t="inlineStr"/>
-      <c r="L159" s="4" t="inlineStr"/>
+      <c r="K159" s="4" t="n">
+        <v>0.9764</v>
+      </c>
+      <c r="L159" s="4" t="n">
+        <v>0.9767</v>
+      </c>
       <c r="M159" s="4" t="n">
-        <v>0.9586</v>
+        <v>0.9751</v>
       </c>
       <c r="N159" s="4" t="n">
-        <v>0.9556</v>
+        <v>0.9823</v>
       </c>
       <c r="O159" s="4" t="inlineStr"/>
       <c r="P159" s="4" t="inlineStr"/>
@@ -9140,12 +9236,12 @@
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>CHBESSG1</t>
+          <t>WDBESSG1</t>
         </is>
       </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
-          <t>Chinchilla BESS</t>
+          <t>Western Downs Battery Energy Storage System (BESS)</t>
         </is>
       </c>
       <c r="C160" s="2" t="inlineStr">
@@ -9154,7 +9250,7 @@
         </is>
       </c>
       <c r="D160" s="3" t="n">
-        <v>134</v>
+        <v>272</v>
       </c>
       <c r="E160" s="4" t="inlineStr"/>
       <c r="F160" s="4" t="inlineStr"/>
@@ -9165,10 +9261,10 @@
       <c r="K160" s="4" t="inlineStr"/>
       <c r="L160" s="4" t="inlineStr"/>
       <c r="M160" s="4" t="n">
-        <v>0.9588</v>
+        <v>0.9586</v>
       </c>
       <c r="N160" s="4" t="n">
-        <v>0.9611</v>
+        <v>0.9556</v>
       </c>
       <c r="O160" s="4" t="inlineStr"/>
       <c r="P160" s="4" t="inlineStr"/>
@@ -9178,12 +9274,12 @@
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>WANDBG1</t>
+          <t>CHBESSG1</t>
         </is>
       </c>
       <c r="B161" s="2" t="inlineStr">
         <is>
-          <t>Wandoan BESS</t>
+          <t>Chinchilla BESS</t>
         </is>
       </c>
       <c r="C161" s="2" t="inlineStr">
@@ -9192,7 +9288,7 @@
         </is>
       </c>
       <c r="D161" s="3" t="n">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="E161" s="4" t="inlineStr"/>
       <c r="F161" s="4" t="inlineStr"/>
@@ -9200,17 +9296,13 @@
       <c r="H161" s="4" t="inlineStr"/>
       <c r="I161" s="4" t="inlineStr"/>
       <c r="J161" s="4" t="inlineStr"/>
-      <c r="K161" s="4" t="n">
-        <v>0.9764</v>
-      </c>
-      <c r="L161" s="4" t="n">
-        <v>0.9767</v>
-      </c>
+      <c r="K161" s="4" t="inlineStr"/>
+      <c r="L161" s="4" t="inlineStr"/>
       <c r="M161" s="4" t="n">
-        <v>0.9751</v>
+        <v>0.9588</v>
       </c>
       <c r="N161" s="4" t="n">
-        <v>0.9823</v>
+        <v>0.9611</v>
       </c>
       <c r="O161" s="4" t="inlineStr"/>
       <c r="P161" s="4" t="inlineStr"/>
@@ -9652,13 +9744,13 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>KSP1</t>
+          <t>HUGSF1</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr"/>
       <c r="C10" s="4" t="inlineStr"/>
       <c r="D10" s="4" t="n">
-        <v>1.0149</v>
+        <v>1.0115</v>
       </c>
       <c r="E10" s="4" t="n">
         <v>0.8842</v>
@@ -9730,13 +9822,13 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>HUGSF1</t>
+          <t>KSP1</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr"/>
       <c r="C12" s="4" t="inlineStr"/>
       <c r="D12" s="4" t="n">
-        <v>1.0115</v>
+        <v>1.0149</v>
       </c>
       <c r="E12" s="4" t="n">
         <v>0.8842</v>
@@ -9868,16 +9960,14 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>LRSF1</t>
+          <t>CLERMSF1</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr"/>
       <c r="C16" s="4" t="inlineStr"/>
-      <c r="D16" s="4" t="n">
-        <v>0.9689</v>
-      </c>
+      <c r="D16" s="4" t="inlineStr"/>
       <c r="E16" s="4" t="n">
-        <v>0.8934</v>
+        <v>0.8862</v>
       </c>
       <c r="F16" s="4" t="n">
         <v>0.8735000000000001</v>
@@ -9948,14 +10038,16 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>CLERMSF1</t>
+          <t>LRSF1</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr"/>
       <c r="C18" s="4" t="inlineStr"/>
-      <c r="D18" s="4" t="inlineStr"/>
+      <c r="D18" s="4" t="n">
+        <v>0.9689</v>
+      </c>
       <c r="E18" s="4" t="n">
-        <v>0.8862</v>
+        <v>0.8934</v>
       </c>
       <c r="F18" s="4" t="n">
         <v>0.8735000000000001</v>
@@ -10105,8 +10197,12 @@
       <c r="H23" s="4" t="inlineStr"/>
       <c r="I23" s="4" t="inlineStr"/>
       <c r="J23" s="4" t="inlineStr"/>
-      <c r="K23" s="4" t="inlineStr"/>
-      <c r="L23" s="4" t="inlineStr"/>
+      <c r="K23" s="4" t="n">
+        <v>0.9528</v>
+      </c>
+      <c r="L23" s="4" t="n">
+        <v>0.9358</v>
+      </c>
       <c r="M23" s="4" t="n">
         <v>0.9008</v>
       </c>
@@ -10329,7 +10425,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>OAKY2</t>
+          <t>OAKYCREK</t>
         </is>
       </c>
       <c r="B29" s="4" t="n">
@@ -10372,7 +10468,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>OAKYCREK</t>
+          <t>OAKY2</t>
         </is>
       </c>
       <c r="B30" s="4" t="n">
@@ -10415,7 +10511,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>CALL_A_4</t>
+          <t>CALLNL4</t>
         </is>
       </c>
       <c r="B31" s="4" t="n">
@@ -10450,7 +10546,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>CALLNL4</t>
+          <t>CALL_A_4</t>
         </is>
       </c>
       <c r="B32" s="4" t="n">
@@ -10485,7 +10581,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>STAN-3</t>
+          <t>STAN-1</t>
         </is>
       </c>
       <c r="B33" s="4" t="n">
@@ -10571,7 +10667,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>STAN-1</t>
+          <t>STAN-3</t>
         </is>
       </c>
       <c r="B35" s="4" t="n">
@@ -10829,7 +10925,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>BRDDSF01</t>
+          <t>BRDDBES1</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr"/>
@@ -10852,7 +10948,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>BRDDBES1</t>
+          <t>BRDDSF01</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr"/>
@@ -10865,7 +10961,9 @@
       <c r="I42" s="4" t="inlineStr"/>
       <c r="J42" s="4" t="inlineStr"/>
       <c r="K42" s="4" t="inlineStr"/>
-      <c r="L42" s="4" t="inlineStr"/>
+      <c r="L42" s="4" t="n">
+        <v>0.929</v>
+      </c>
       <c r="M42" s="4" t="n">
         <v>0.9247</v>
       </c>
@@ -11045,7 +11143,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>GSTONE6</t>
+          <t>GSTONE5</t>
         </is>
       </c>
       <c r="B47" s="4" t="n">
@@ -11088,7 +11186,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>GSTONE5</t>
+          <t>GSTONE6</t>
         </is>
       </c>
       <c r="B48" s="4" t="n">
@@ -11510,7 +11608,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>SRSF1</t>
+          <t>CHILDSF1</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr"/>
@@ -11547,7 +11645,7 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>CHILDSF1</t>
+          <t>SRSF1</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr"/>
@@ -11627,7 +11725,7 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>MSTUART3</t>
+          <t>MSTUART2</t>
         </is>
       </c>
       <c r="B63" s="4" t="n">
@@ -11670,7 +11768,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>MSTUART2</t>
+          <t>MSTUART3</t>
         </is>
       </c>
       <c r="B64" s="4" t="n">
@@ -11887,7 +11985,7 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>KAREEYA4</t>
+          <t>KAREEYA2</t>
         </is>
       </c>
       <c r="B71" s="4" t="n">
@@ -11930,7 +12028,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>KAREEYA1</t>
+          <t>KAREEYA5</t>
         </is>
       </c>
       <c r="B72" s="4" t="n">
@@ -11973,7 +12071,7 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>KAREEYA2</t>
+          <t>KAREEYA4</t>
         </is>
       </c>
       <c r="B73" s="4" t="n">
@@ -12059,7 +12157,7 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>KAREEYA5</t>
+          <t>KAREEYA1</t>
         </is>
       </c>
       <c r="B75" s="4" t="n">
@@ -12293,7 +12391,7 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>BRAEMAR6</t>
+          <t>BRAEMAR2</t>
         </is>
       </c>
       <c r="B81" s="4" t="n">
@@ -12379,7 +12477,7 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>BRAEMAR1</t>
+          <t>BRAEMAR7</t>
         </is>
       </c>
       <c r="B83" s="4" t="n">
@@ -12422,7 +12520,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>BRAEMAR2</t>
+          <t>BRAEMAR6</t>
         </is>
       </c>
       <c r="B84" s="4" t="n">
@@ -12465,7 +12563,7 @@
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>BRAEMAR7</t>
+          <t>BRAEMAR1</t>
         </is>
       </c>
       <c r="B85" s="4" t="n">
@@ -12662,7 +12760,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>TARONG#4</t>
+          <t>TARONG#3</t>
         </is>
       </c>
       <c r="B90" s="4" t="n">
@@ -12705,7 +12803,7 @@
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>TARONG#3</t>
+          <t>TARONG#4</t>
         </is>
       </c>
       <c r="B91" s="4" t="n">
@@ -12963,8 +13061,12 @@
       <c r="H97" s="4" t="inlineStr"/>
       <c r="I97" s="4" t="inlineStr"/>
       <c r="J97" s="4" t="inlineStr"/>
-      <c r="K97" s="4" t="inlineStr"/>
-      <c r="L97" s="4" t="inlineStr"/>
+      <c r="K97" s="4" t="n">
+        <v>0.9837</v>
+      </c>
+      <c r="L97" s="4" t="n">
+        <v>0.9836</v>
+      </c>
       <c r="M97" s="4" t="n">
         <v>0.9772999999999999</v>
       </c>
@@ -13015,7 +13117,7 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>ROMA_7</t>
+          <t>ROMA_8</t>
         </is>
       </c>
       <c r="B99" s="4" t="n">
@@ -13058,7 +13160,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>ROMA_8</t>
+          <t>ROMA_7</t>
         </is>
       </c>
       <c r="B100" s="4" t="n">
@@ -13113,8 +13215,12 @@
       <c r="H101" s="4" t="inlineStr"/>
       <c r="I101" s="4" t="inlineStr"/>
       <c r="J101" s="4" t="inlineStr"/>
-      <c r="K101" s="4" t="inlineStr"/>
-      <c r="L101" s="4" t="inlineStr"/>
+      <c r="K101" s="4" t="n">
+        <v>0.9698</v>
+      </c>
+      <c r="L101" s="4" t="n">
+        <v>0.9851</v>
+      </c>
       <c r="M101" s="4" t="n">
         <v>0.9778</v>
       </c>
@@ -13134,8 +13240,12 @@
       <c r="H102" s="4" t="inlineStr"/>
       <c r="I102" s="4" t="inlineStr"/>
       <c r="J102" s="4" t="inlineStr"/>
-      <c r="K102" s="4" t="inlineStr"/>
-      <c r="L102" s="4" t="inlineStr"/>
+      <c r="K102" s="4" t="n">
+        <v>0.9761</v>
+      </c>
+      <c r="L102" s="4" t="n">
+        <v>0.9875</v>
+      </c>
       <c r="M102" s="4" t="n">
         <v>0.9787</v>
       </c>
@@ -13406,7 +13516,7 @@
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>WDBESS1</t>
+          <t>WDBESS2</t>
         </is>
       </c>
       <c r="B110" s="4" t="inlineStr"/>
@@ -13419,7 +13529,9 @@
       <c r="I110" s="4" t="inlineStr"/>
       <c r="J110" s="4" t="inlineStr"/>
       <c r="K110" s="4" t="inlineStr"/>
-      <c r="L110" s="4" t="inlineStr"/>
+      <c r="L110" s="4" t="n">
+        <v>0.9899</v>
+      </c>
       <c r="M110" s="4" t="n">
         <v>0.9801</v>
       </c>
@@ -13427,7 +13539,7 @@
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>WDBESS2</t>
+          <t>WDBESS1</t>
         </is>
       </c>
       <c r="B111" s="4" t="inlineStr"/>
@@ -13439,8 +13551,12 @@
       <c r="H111" s="4" t="inlineStr"/>
       <c r="I111" s="4" t="inlineStr"/>
       <c r="J111" s="4" t="inlineStr"/>
-      <c r="K111" s="4" t="inlineStr"/>
-      <c r="L111" s="4" t="inlineStr"/>
+      <c r="K111" s="4" t="n">
+        <v>0.9762</v>
+      </c>
+      <c r="L111" s="4" t="n">
+        <v>0.9891</v>
+      </c>
       <c r="M111" s="4" t="n">
         <v>0.9801</v>
       </c>
@@ -13734,27 +13850,33 @@
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>DULAWF1</t>
+          <t>MARYRSF1</t>
         </is>
       </c>
       <c r="B120" s="4" t="inlineStr"/>
       <c r="C120" s="4" t="inlineStr"/>
       <c r="D120" s="4" t="inlineStr"/>
       <c r="E120" s="4" t="inlineStr"/>
-      <c r="F120" s="4" t="inlineStr"/>
-      <c r="G120" s="4" t="inlineStr"/>
-      <c r="H120" s="4" t="inlineStr"/>
+      <c r="F120" s="4" t="n">
+        <v>0.9872</v>
+      </c>
+      <c r="G120" s="4" t="n">
+        <v>0.9851</v>
+      </c>
+      <c r="H120" s="4" t="n">
+        <v>0.9789</v>
+      </c>
       <c r="I120" s="4" t="n">
-        <v>0.9540999999999999</v>
+        <v>0.9861</v>
       </c>
       <c r="J120" s="4" t="n">
-        <v>0.9776</v>
+        <v>0.9913999999999999</v>
       </c>
       <c r="K120" s="4" t="n">
-        <v>0.977</v>
+        <v>0.9847</v>
       </c>
       <c r="L120" s="4" t="n">
-        <v>0.9853</v>
+        <v>0.9888</v>
       </c>
       <c r="M120" s="4" t="n">
         <v>0.987</v>
@@ -13763,16 +13885,14 @@
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>MARYRSF1</t>
+          <t>WARWSF1</t>
         </is>
       </c>
       <c r="B121" s="4" t="inlineStr"/>
       <c r="C121" s="4" t="inlineStr"/>
       <c r="D121" s="4" t="inlineStr"/>
       <c r="E121" s="4" t="inlineStr"/>
-      <c r="F121" s="4" t="n">
-        <v>0.9872</v>
-      </c>
+      <c r="F121" s="4" t="inlineStr"/>
       <c r="G121" s="4" t="n">
         <v>0.9851</v>
       </c>
@@ -13798,7 +13918,7 @@
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>WARWSF1</t>
+          <t>DULAWF1</t>
         </is>
       </c>
       <c r="B122" s="4" t="inlineStr"/>
@@ -13806,23 +13926,19 @@
       <c r="D122" s="4" t="inlineStr"/>
       <c r="E122" s="4" t="inlineStr"/>
       <c r="F122" s="4" t="inlineStr"/>
-      <c r="G122" s="4" t="n">
-        <v>0.9851</v>
-      </c>
-      <c r="H122" s="4" t="n">
-        <v>0.9789</v>
-      </c>
+      <c r="G122" s="4" t="inlineStr"/>
+      <c r="H122" s="4" t="inlineStr"/>
       <c r="I122" s="4" t="n">
-        <v>0.9861</v>
+        <v>0.9540999999999999</v>
       </c>
       <c r="J122" s="4" t="n">
-        <v>0.9913999999999999</v>
+        <v>0.9776</v>
       </c>
       <c r="K122" s="4" t="n">
-        <v>0.9847</v>
+        <v>0.977</v>
       </c>
       <c r="L122" s="4" t="n">
-        <v>0.9888</v>
+        <v>0.9853</v>
       </c>
       <c r="M122" s="4" t="n">
         <v>0.987</v>
@@ -14055,20 +14171,42 @@
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>SNB02</t>
-        </is>
-      </c>
-      <c r="B129" s="4" t="inlineStr"/>
-      <c r="C129" s="4" t="inlineStr"/>
-      <c r="D129" s="4" t="inlineStr"/>
-      <c r="E129" s="4" t="inlineStr"/>
-      <c r="F129" s="4" t="inlineStr"/>
-      <c r="G129" s="4" t="inlineStr"/>
-      <c r="H129" s="4" t="inlineStr"/>
-      <c r="I129" s="4" t="inlineStr"/>
-      <c r="J129" s="4" t="inlineStr"/>
-      <c r="K129" s="4" t="inlineStr"/>
-      <c r="L129" s="4" t="inlineStr"/>
+          <t>DG_QLD1</t>
+        </is>
+      </c>
+      <c r="B129" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C129" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D129" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E129" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F129" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G129" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H129" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I129" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J129" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K129" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L129" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="M129" s="4" t="n">
         <v>1</v>
       </c>
@@ -14088,8 +14226,12 @@
       <c r="H130" s="4" t="inlineStr"/>
       <c r="I130" s="4" t="inlineStr"/>
       <c r="J130" s="4" t="inlineStr"/>
-      <c r="K130" s="4" t="inlineStr"/>
-      <c r="L130" s="4" t="inlineStr"/>
+      <c r="K130" s="4" t="n">
+        <v>0.9877</v>
+      </c>
+      <c r="L130" s="4" t="n">
+        <v>1.0066</v>
+      </c>
       <c r="M130" s="4" t="n">
         <v>1</v>
       </c>
@@ -14097,39 +14239,19 @@
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>DG_QLD1</t>
-        </is>
-      </c>
-      <c r="B131" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C131" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D131" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E131" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F131" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G131" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H131" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I131" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J131" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K131" s="4" t="n">
-        <v>1</v>
-      </c>
+          <t>SNB02</t>
+        </is>
+      </c>
+      <c r="B131" s="4" t="inlineStr"/>
+      <c r="C131" s="4" t="inlineStr"/>
+      <c r="D131" s="4" t="inlineStr"/>
+      <c r="E131" s="4" t="inlineStr"/>
+      <c r="F131" s="4" t="inlineStr"/>
+      <c r="G131" s="4" t="inlineStr"/>
+      <c r="H131" s="4" t="inlineStr"/>
+      <c r="I131" s="4" t="inlineStr"/>
+      <c r="J131" s="4" t="inlineStr"/>
+      <c r="K131" s="4" t="inlineStr"/>
       <c r="L131" s="4" t="n">
         <v>1</v>
       </c>
@@ -14153,7 +14275,9 @@
       <c r="I132" s="4" t="inlineStr"/>
       <c r="J132" s="4" t="inlineStr"/>
       <c r="K132" s="4" t="inlineStr"/>
-      <c r="L132" s="4" t="inlineStr"/>
+      <c r="L132" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="M132" s="4" t="n">
         <v>1</v>
       </c>
@@ -14259,7 +14383,9 @@
       <c r="I136" s="4" t="inlineStr"/>
       <c r="J136" s="4" t="inlineStr"/>
       <c r="K136" s="4" t="inlineStr"/>
-      <c r="L136" s="4" t="inlineStr"/>
+      <c r="L136" s="4" t="n">
+        <v>1.0036</v>
+      </c>
       <c r="M136" s="4" t="n">
         <v>1.0015</v>
       </c>
@@ -14366,7 +14492,9 @@
       <c r="I139" s="4" t="inlineStr"/>
       <c r="J139" s="4" t="inlineStr"/>
       <c r="K139" s="4" t="inlineStr"/>
-      <c r="L139" s="4" t="inlineStr"/>
+      <c r="L139" s="4" t="n">
+        <v>1.0014</v>
+      </c>
       <c r="M139" s="4" t="n">
         <v>1.0027</v>
       </c>
@@ -14429,8 +14557,12 @@
       <c r="H141" s="4" t="inlineStr"/>
       <c r="I141" s="4" t="inlineStr"/>
       <c r="J141" s="4" t="inlineStr"/>
-      <c r="K141" s="4" t="inlineStr"/>
-      <c r="L141" s="4" t="inlineStr"/>
+      <c r="K141" s="4" t="n">
+        <v>1.0033</v>
+      </c>
+      <c r="L141" s="4" t="n">
+        <v>1.0045</v>
+      </c>
       <c r="M141" s="4" t="n">
         <v>1.0035</v>
       </c>
@@ -14481,15 +14613,11 @@
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>RPCG</t>
-        </is>
-      </c>
-      <c r="B143" s="4" t="n">
-        <v>1.0078</v>
-      </c>
-      <c r="C143" s="4" t="n">
-        <v>1.008</v>
-      </c>
+          <t>STAPYLTON1</t>
+        </is>
+      </c>
+      <c r="B143" s="4" t="inlineStr"/>
+      <c r="C143" s="4" t="inlineStr"/>
       <c r="D143" s="4" t="n">
         <v>1.0112</v>
       </c>
@@ -14524,11 +14652,15 @@
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>STAPYLTON1</t>
-        </is>
-      </c>
-      <c r="B144" s="4" t="inlineStr"/>
-      <c r="C144" s="4" t="inlineStr"/>
+          <t>RPCG</t>
+        </is>
+      </c>
+      <c r="B144" s="4" t="n">
+        <v>1.0078</v>
+      </c>
+      <c r="C144" s="4" t="n">
+        <v>1.008</v>
+      </c>
       <c r="D144" s="4" t="n">
         <v>1.0112</v>
       </c>
@@ -14837,23 +14969,23 @@
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>EDLRGNRD</t>
+          <t>ROCHEDAL</t>
         </is>
       </c>
       <c r="B153" s="4" t="n">
-        <v>1.0057</v>
+        <v>1.0067</v>
       </c>
       <c r="C153" s="4" t="n">
-        <v>1.0049</v>
+        <v>1.0091</v>
       </c>
       <c r="D153" s="4" t="n">
-        <v>1.0044</v>
+        <v>1.0114</v>
       </c>
       <c r="E153" s="4" t="n">
-        <v>1.0042</v>
+        <v>1.0123</v>
       </c>
       <c r="F153" s="4" t="n">
-        <v>1.0042</v>
+        <v>1.0121</v>
       </c>
       <c r="G153" s="4" t="inlineStr"/>
       <c r="H153" s="4" t="inlineStr"/>
@@ -14866,23 +14998,23 @@
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>ROCHEDAL</t>
+          <t>WHIT1</t>
         </is>
       </c>
       <c r="B154" s="4" t="n">
-        <v>1.0067</v>
+        <v>0.9953</v>
       </c>
       <c r="C154" s="4" t="n">
-        <v>1.0091</v>
+        <v>0.9968</v>
       </c>
       <c r="D154" s="4" t="n">
-        <v>1.0114</v>
+        <v>0.9999</v>
       </c>
       <c r="E154" s="4" t="n">
-        <v>1.0123</v>
+        <v>1.0001</v>
       </c>
       <c r="F154" s="4" t="n">
-        <v>1.0121</v>
+        <v>1.0006</v>
       </c>
       <c r="G154" s="4" t="inlineStr"/>
       <c r="H154" s="4" t="inlineStr"/>
@@ -14895,23 +15027,23 @@
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>WHIT1</t>
+          <t>EDLRGNRD</t>
         </is>
       </c>
       <c r="B155" s="4" t="n">
-        <v>0.9953</v>
+        <v>1.0057</v>
       </c>
       <c r="C155" s="4" t="n">
-        <v>0.9968</v>
+        <v>1.0049</v>
       </c>
       <c r="D155" s="4" t="n">
-        <v>0.9999</v>
+        <v>1.0044</v>
       </c>
       <c r="E155" s="4" t="n">
-        <v>1.0001</v>
+        <v>1.0042</v>
       </c>
       <c r="F155" s="4" t="n">
-        <v>1.0006</v>
+        <v>1.0042</v>
       </c>
       <c r="G155" s="4" t="inlineStr"/>
       <c r="H155" s="4" t="inlineStr"/>
@@ -15025,7 +15157,7 @@
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>WDBESSG1</t>
+          <t>WANDBG1</t>
         </is>
       </c>
       <c r="B159" s="4" t="inlineStr"/>
@@ -15034,13 +15166,17 @@
       <c r="E159" s="4" t="inlineStr"/>
       <c r="F159" s="4" t="inlineStr"/>
       <c r="G159" s="4" t="inlineStr"/>
-      <c r="H159" s="4" t="inlineStr"/>
-      <c r="I159" s="4" t="inlineStr"/>
+      <c r="H159" s="4" t="n">
+        <v>0.9764</v>
+      </c>
+      <c r="I159" s="4" t="n">
+        <v>0.9767</v>
+      </c>
       <c r="J159" s="4" t="n">
-        <v>0.9586</v>
+        <v>0.9751</v>
       </c>
       <c r="K159" s="4" t="n">
-        <v>0.9556</v>
+        <v>0.9823</v>
       </c>
       <c r="L159" s="4" t="inlineStr"/>
       <c r="M159" s="4" t="inlineStr"/>
@@ -15048,7 +15184,7 @@
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>CHBESSG1</t>
+          <t>WDBESSG1</t>
         </is>
       </c>
       <c r="B160" s="4" t="inlineStr"/>
@@ -15060,10 +15196,10 @@
       <c r="H160" s="4" t="inlineStr"/>
       <c r="I160" s="4" t="inlineStr"/>
       <c r="J160" s="4" t="n">
-        <v>0.9588</v>
+        <v>0.9586</v>
       </c>
       <c r="K160" s="4" t="n">
-        <v>0.9611</v>
+        <v>0.9556</v>
       </c>
       <c r="L160" s="4" t="inlineStr"/>
       <c r="M160" s="4" t="inlineStr"/>
@@ -15071,7 +15207,7 @@
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>WANDBG1</t>
+          <t>CHBESSG1</t>
         </is>
       </c>
       <c r="B161" s="4" t="inlineStr"/>
@@ -15080,17 +15216,13 @@
       <c r="E161" s="4" t="inlineStr"/>
       <c r="F161" s="4" t="inlineStr"/>
       <c r="G161" s="4" t="inlineStr"/>
-      <c r="H161" s="4" t="n">
-        <v>0.9764</v>
-      </c>
-      <c r="I161" s="4" t="n">
-        <v>0.9767</v>
-      </c>
+      <c r="H161" s="4" t="inlineStr"/>
+      <c r="I161" s="4" t="inlineStr"/>
       <c r="J161" s="4" t="n">
-        <v>0.9751</v>
+        <v>0.9588</v>
       </c>
       <c r="K161" s="4" t="n">
-        <v>0.9823</v>
+        <v>0.9611</v>
       </c>
       <c r="L161" s="4" t="inlineStr"/>
       <c r="M161" s="4" t="inlineStr"/>
@@ -15477,12 +15609,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>HUGSF1</t>
+          <t>KSP1</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Hughenden Solar Farm</t>
+          <t>Kidston Solar Project Phase One</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -15506,12 +15638,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>KSP1</t>
+          <t>HUGSF1</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Kidston Solar Project Phase One</t>
+          <t>Hughenden Solar Farm</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -15767,12 +15899,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>LRSF1</t>
+          <t>CLERMSF1</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Longreach Solar Farm</t>
+          <t>Clermont Solar Farm</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -15796,12 +15928,12 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>CLERMSF1</t>
+          <t>LRSF1</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Clermont Solar Farm</t>
+          <t>Longreach Solar Farm</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -15985,7 +16117,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>MSTUART3</t>
+          <t>MSTUART2</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -16014,7 +16146,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>MSTUART2</t>
+          <t>MSTUART3</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -16159,7 +16291,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>ROMA_7</t>
+          <t>ROMA_8</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -16188,7 +16320,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>ROMA_8</t>
+          <t>ROMA_7</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -16246,12 +16378,12 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>BRAEMAR2</t>
+          <t>BRAEMAR6</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Braemar Power Station</t>
+          <t>Braemar 2 Power Station</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -16275,12 +16407,12 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>BRAEMAR1</t>
+          <t>BRAEMAR7</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Braemar Power Station</t>
+          <t>Braemar 2 Power Station</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -16304,12 +16436,12 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>BRAEMAR7</t>
+          <t>BRAEMAR1</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Braemar 2 Power Station</t>
+          <t>Braemar Power Station</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -16333,12 +16465,12 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>BRAEMAR6</t>
+          <t>BRAEMAR2</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Braemar 2 Power Station</t>
+          <t>Braemar Power Station</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -16507,12 +16639,12 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>RPCG</t>
+          <t>STAPYLTON1</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Rocky Point Cogeneration Plant</t>
+          <t>Stapylton Renewable Energy Facility</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">

</xml_diff>